<commit_message>
Add live Overall formula column to proa_scraped.xlsx
Weights on a _Overall_Model sheet, generated from overall_model.json by overall_sheet.py (also run by fit_overall and the scraper).

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/proa_scraped.xlsx
+++ b/proa_scraped.xlsx
@@ -25,6 +25,7 @@
     <sheet name="Wolmirstedt" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Tubingen" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="Stars Bochum" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="_Overall_Model" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,13 +35,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -63,8 +67,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,8 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF16"/>
+  <dimension ref="A1:AG16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -594,6 +602,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -697,6 +710,10 @@
       <c r="AF2" t="n">
         <v>2005105</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -800,6 +817,10 @@
       <c r="AF3" t="n">
         <v>2004392</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -903,6 +924,10 @@
       <c r="AF4" t="n">
         <v>2000116</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1006,6 +1031,10 @@
       <c r="AF5" t="n">
         <v>2001880</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1109,6 +1138,10 @@
       <c r="AF6" t="n">
         <v>2001879</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1212,6 +1245,10 @@
       <c r="AF7" t="n">
         <v>1400019</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1315,6 +1352,10 @@
       <c r="AF8" t="n">
         <v>2004440</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1418,6 +1459,10 @@
       <c r="AF9" t="n">
         <v>2005245</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1521,6 +1566,10 @@
       <c r="AF10" t="n">
         <v>2004414</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1624,6 +1673,10 @@
       <c r="AF11" t="n">
         <v>2001690</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1727,6 +1780,10 @@
       <c r="AF12" t="n">
         <v>2004438</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1830,6 +1887,10 @@
       <c r="AF13" t="n">
         <v>2004622</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1933,6 +1994,10 @@
       <c r="AF14" t="n">
         <v>2003111</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2036,6 +2101,10 @@
       <c r="AF15" t="n">
         <v>2002110</v>
       </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2138,6 +2207,10 @@
       </c>
       <c r="AF16" t="n">
         <v>2004604</v>
+      </c>
+      <c r="AG16">
+        <f>IF(ISNA(MATCH($C16,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L16:AD16,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*IF(Q16&gt;=75,99,IF(Q16&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*J16+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*K16,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2151,8 +2224,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF16"/>
+  <dimension ref="A1:AG16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2315,6 +2391,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2418,6 +2499,10 @@
       <c r="AF2" t="n">
         <v>1400013</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2521,6 +2606,10 @@
       <c r="AF3" t="n">
         <v>2003953</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2624,6 +2713,10 @@
       <c r="AF4" t="n">
         <v>2005080</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2727,6 +2820,10 @@
       <c r="AF5" t="n">
         <v>2003787</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2830,6 +2927,10 @@
       <c r="AF6" t="n">
         <v>2003788</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2933,6 +3034,10 @@
       <c r="AF7" t="n">
         <v>2003786</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3036,6 +3141,10 @@
       <c r="AF8" t="n">
         <v>56479</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3139,6 +3248,10 @@
       <c r="AF9" t="n">
         <v>1000853</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3242,6 +3355,10 @@
       <c r="AF10" t="n">
         <v>2001528</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3345,6 +3462,10 @@
       <c r="AF11" t="n">
         <v>2003954</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3448,6 +3569,10 @@
       <c r="AF12" t="n">
         <v>56380</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3551,6 +3676,10 @@
       <c r="AF13" t="n">
         <v>2004391</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3654,6 +3783,10 @@
       <c r="AF14" t="n">
         <v>2004146</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3757,6 +3890,10 @@
       <c r="AF15" t="n">
         <v>2004390</v>
       </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3859,6 +3996,10 @@
       </c>
       <c r="AF16" t="n">
         <v>2004007</v>
+      </c>
+      <c r="AG16">
+        <f>IF(ISNA(MATCH($C16,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L16:AD16,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*IF(Q16&gt;=75,99,IF(Q16&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*J16+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*K16,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3872,8 +4013,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF16"/>
+  <dimension ref="A1:AG16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4036,6 +4180,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4139,6 +4288,10 @@
       <c r="AF2" t="n">
         <v>2004101</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4242,6 +4395,10 @@
       <c r="AF3" t="n">
         <v>2004048</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4345,6 +4502,10 @@
       <c r="AF4" t="n">
         <v>2004046</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4448,6 +4609,10 @@
       <c r="AF5" t="n">
         <v>5034</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4551,6 +4716,10 @@
       <c r="AF6" t="n">
         <v>2004435</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4654,6 +4823,10 @@
       <c r="AF7" t="n">
         <v>5469</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4757,6 +4930,10 @@
       <c r="AF8" t="n">
         <v>2001468</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4860,6 +5037,10 @@
       <c r="AF9" t="n">
         <v>2003981</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4963,6 +5144,10 @@
       <c r="AF10" t="n">
         <v>2004965</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5066,6 +5251,10 @@
       <c r="AF11" t="n">
         <v>2003982</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5169,6 +5358,10 @@
       <c r="AF12" t="n">
         <v>2003983</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5272,6 +5465,10 @@
       <c r="AF13" t="n">
         <v>2001806</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5375,6 +5572,10 @@
       <c r="AF14" t="n">
         <v>2004606</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5478,6 +5679,10 @@
       <c r="AF15" t="n">
         <v>58183</v>
       </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5580,6 +5785,10 @@
       </c>
       <c r="AF16" t="n">
         <v>2003104</v>
+      </c>
+      <c r="AG16">
+        <f>IF(ISNA(MATCH($C16,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L16:AD16,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*IF(Q16&gt;=75,99,IF(Q16&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*J16+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*K16,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -5593,8 +5802,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF16"/>
+  <dimension ref="A1:AG16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -5757,6 +5969,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5860,6 +6077,10 @@
       <c r="AF2" t="n">
         <v>2004110</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5963,6 +6184,10 @@
       <c r="AF3" t="n">
         <v>2004602</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6066,6 +6291,10 @@
       <c r="AF4" t="n">
         <v>2005115</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6169,6 +6398,10 @@
       <c r="AF5" t="n">
         <v>2001946</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6272,6 +6505,10 @@
       <c r="AF6" t="n">
         <v>2001368</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6375,6 +6612,10 @@
       <c r="AF7" t="n">
         <v>2000160</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6478,6 +6719,10 @@
       <c r="AF8" t="n">
         <v>2004513</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6581,6 +6826,10 @@
       <c r="AF9" t="n">
         <v>2001259</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6684,6 +6933,10 @@
       <c r="AF10" t="n">
         <v>2001947</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6787,6 +7040,10 @@
       <c r="AF11" t="n">
         <v>2005025</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6890,6 +7147,10 @@
       <c r="AF12" t="n">
         <v>2004525</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6993,6 +7254,10 @@
       <c r="AF13" t="n">
         <v>2004163</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7096,6 +7361,10 @@
       <c r="AF14" t="n">
         <v>2001363</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7199,6 +7468,10 @@
       <c r="AF15" t="n">
         <v>2001951</v>
       </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7301,6 +7574,10 @@
       </c>
       <c r="AF16" t="n">
         <v>2002104</v>
+      </c>
+      <c r="AG16">
+        <f>IF(ISNA(MATCH($C16,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L16:AD16,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*IF(Q16&gt;=75,99,IF(Q16&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*J16+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*K16,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -7314,8 +7591,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF13"/>
+  <dimension ref="A1:AG13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -7478,6 +7758,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7581,6 +7866,10 @@
       <c r="AF2" t="n">
         <v>2004481</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7684,6 +7973,10 @@
       <c r="AF3" t="n">
         <v>2004483</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7787,6 +8080,10 @@
       <c r="AF4" t="n">
         <v>2004480</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7890,6 +8187,10 @@
       <c r="AF5" t="n">
         <v>2005106</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7993,6 +8294,10 @@
       <c r="AF6" t="n">
         <v>2004482</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8096,6 +8401,10 @@
       <c r="AF7" t="n">
         <v>2004484</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8199,6 +8508,10 @@
       <c r="AF8" t="n">
         <v>6272</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8302,6 +8615,10 @@
       <c r="AF9" t="n">
         <v>2002140</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8405,6 +8722,10 @@
       <c r="AF10" t="n">
         <v>2001051</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8508,6 +8829,10 @@
       <c r="AF11" t="n">
         <v>2004485</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8611,6 +8936,10 @@
       <c r="AF12" t="n">
         <v>2005108</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8713,6 +9042,10 @@
       </c>
       <c r="AF13" t="n">
         <v>2005107</v>
+      </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -8726,8 +9059,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF15"/>
+  <dimension ref="A1:AG15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8890,6 +9226,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8993,6 +9334,10 @@
       <c r="AF2" t="n">
         <v>2004016</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9096,6 +9441,10 @@
       <c r="AF3" t="n">
         <v>2003099</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9199,6 +9548,10 @@
       <c r="AF4" t="n">
         <v>2004189</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9302,6 +9655,10 @@
       <c r="AF5" t="n">
         <v>2001526</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9405,6 +9762,10 @@
       <c r="AF6" t="n">
         <v>2004014</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9508,6 +9869,10 @@
       <c r="AF7" t="n">
         <v>2001572</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9611,6 +9976,10 @@
       <c r="AF8" t="n">
         <v>2001322</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9714,6 +10083,10 @@
       <c r="AF9" t="n">
         <v>2004017</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9817,6 +10190,10 @@
       <c r="AF10" t="n">
         <v>1400015</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9920,6 +10297,10 @@
       <c r="AF11" t="n">
         <v>2005310</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -10023,6 +10404,10 @@
       <c r="AF12" t="n">
         <v>2004187</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -10126,6 +10511,10 @@
       <c r="AF13" t="n">
         <v>2002947</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -10229,6 +10618,10 @@
       <c r="AF14" t="n">
         <v>2004451</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -10331,6 +10724,10 @@
       </c>
       <c r="AF15" t="n">
         <v>2004188</v>
+      </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -10344,8 +10741,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF14"/>
+  <dimension ref="A1:AG14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -10508,6 +10908,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -10611,6 +11016,10 @@
       <c r="AF2" t="n">
         <v>2001447</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10714,6 +11123,10 @@
       <c r="AF3" t="n">
         <v>2002277</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10817,6 +11230,10 @@
       <c r="AF4" t="n">
         <v>2004252</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10920,6 +11337,10 @@
       <c r="AF5" t="n">
         <v>2004249</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11023,6 +11444,10 @@
       <c r="AF6" t="n">
         <v>2004250</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11126,6 +11551,10 @@
       <c r="AF7" t="n">
         <v>2004254</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11229,6 +11658,10 @@
       <c r="AF8" t="n">
         <v>1400017</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11332,6 +11765,10 @@
       <c r="AF9" t="n">
         <v>2001838</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11435,6 +11872,10 @@
       <c r="AF10" t="n">
         <v>57948</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11538,6 +11979,10 @@
       <c r="AF11" t="n">
         <v>2002188</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11641,6 +12086,10 @@
       <c r="AF12" t="n">
         <v>2001841</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11744,6 +12193,10 @@
       <c r="AF13" t="n">
         <v>58073</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11846,6 +12299,10 @@
       </c>
       <c r="AF14" t="n">
         <v>2002994</v>
+      </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -11859,8 +12316,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF15"/>
+  <dimension ref="A1:AG15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -12023,6 +12483,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -12126,6 +12591,10 @@
       <c r="AF2" t="n">
         <v>2004426</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -12229,6 +12698,10 @@
       <c r="AF3" t="n">
         <v>2004201</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12332,6 +12805,10 @@
       <c r="AF4" t="n">
         <v>2004203</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12435,6 +12912,10 @@
       <c r="AF5" t="n">
         <v>2005027</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12538,6 +13019,10 @@
       <c r="AF6" t="n">
         <v>2004206</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12641,6 +13126,10 @@
       <c r="AF7" t="n">
         <v>2004202</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12744,6 +13233,10 @@
       <c r="AF8" t="n">
         <v>5575</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12847,6 +13340,10 @@
       <c r="AF9" t="n">
         <v>2001705</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12950,6 +13447,10 @@
       <c r="AF10" t="n">
         <v>2004200</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13053,6 +13554,10 @@
       <c r="AF11" t="n">
         <v>2004707</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13156,6 +13661,10 @@
       <c r="AF12" t="n">
         <v>2004266</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13259,6 +13768,10 @@
       <c r="AF13" t="n">
         <v>2004199</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13362,6 +13875,10 @@
       <c r="AF14" t="n">
         <v>6055</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13464,6 +13981,10 @@
       </c>
       <c r="AF15" t="n">
         <v>2004267</v>
+      </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -13477,8 +13998,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF16"/>
+  <dimension ref="A1:AG16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -13641,6 +14165,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -13744,6 +14273,10 @@
       <c r="AF2" t="n">
         <v>2003150</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -13847,6 +14380,10 @@
       <c r="AF3" t="n">
         <v>2003819</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -13950,6 +14487,10 @@
       <c r="AF4" t="n">
         <v>2003146</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14053,6 +14594,10 @@
       <c r="AF5" t="n">
         <v>1400000</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14156,6 +14701,10 @@
       <c r="AF6" t="n">
         <v>2004210</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14259,6 +14808,10 @@
       <c r="AF7" t="n">
         <v>2003143</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -14362,6 +14915,10 @@
       <c r="AF8" t="n">
         <v>2000371</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -14465,6 +15022,10 @@
       <c r="AF9" t="n">
         <v>2004990</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -14568,6 +15129,10 @@
       <c r="AF10" t="n">
         <v>2003798</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -14671,6 +15236,10 @@
       <c r="AF11" t="n">
         <v>1400004</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -14774,6 +15343,10 @@
       <c r="AF12" t="n">
         <v>2004237</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14877,6 +15450,10 @@
       <c r="AF13" t="n">
         <v>2004234</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14980,6 +15557,10 @@
       <c r="AF14" t="n">
         <v>2004239</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -15083,6 +15664,10 @@
       <c r="AF15" t="n">
         <v>56773</v>
       </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15185,6 +15770,10 @@
       </c>
       <c r="AF16" t="n">
         <v>2003945</v>
+      </c>
+      <c r="AG16">
+        <f>IF(ISNA(MATCH($C16,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L16:AD16,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*IF(Q16&gt;=75,99,IF(Q16&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*J16+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*K16,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -15198,8 +15787,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF15"/>
+  <dimension ref="A1:AG15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -15362,6 +15954,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -15465,6 +16062,10 @@
       <c r="AF2" t="n">
         <v>2004916</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -15568,6 +16169,10 @@
       <c r="AF3" t="n">
         <v>5119</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15671,6 +16276,10 @@
       <c r="AF4" t="n">
         <v>2004918</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15774,6 +16383,10 @@
       <c r="AF5" t="n">
         <v>2004917</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -15877,6 +16490,10 @@
       <c r="AF6" t="n">
         <v>2003097</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -15980,6 +16597,10 @@
       <c r="AF7" t="n">
         <v>2004907</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -16083,6 +16704,10 @@
       <c r="AF8" t="n">
         <v>5117</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -16186,6 +16811,10 @@
       <c r="AF9" t="n">
         <v>2004915</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -16289,6 +16918,10 @@
       <c r="AF10" t="n">
         <v>2004913</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -16392,6 +17025,10 @@
       <c r="AF11" t="n">
         <v>2004927</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -16495,6 +17132,10 @@
       <c r="AF12" t="n">
         <v>2004928</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -16598,6 +17239,10 @@
       <c r="AF13" t="n">
         <v>2001926</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -16701,6 +17346,10 @@
       <c r="AF14" t="n">
         <v>2004914</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -16803,6 +17452,580 @@
       </c>
       <c r="AF15" t="n">
         <v>2005196</v>
+      </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Close Shot</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Midrange Shot</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>3pt Shot</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Free Throws</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Layup</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Dunk</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Ball Handling</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Post Offense</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Post Defense</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Block</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Steal</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Offensive Rebound</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Defensive Rebound</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Stamina</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Durability</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Defensive Awareness</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Offensive Awareness</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Intercept</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>DunkFlag weight</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Height coef (per m)</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Weight coef (per kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.0503</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.2263</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.0838</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0294</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1129</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0251</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.1293</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1482</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0224</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.0429</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0236</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.1153</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.0615</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.0561</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.0515</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.0238</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.0116</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.0871</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.0759</v>
+      </c>
+      <c r="U2" t="n">
+        <v>-24.9705</v>
+      </c>
+      <c r="V2" t="n">
+        <v>-0.0017</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.2107</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0982</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0941</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.0948</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.1093</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.0572</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.0227</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.0505</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0269</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.0536</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.0459</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.0607</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.06320000000000001</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>-0.0032</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.0853</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0631</v>
+      </c>
+      <c r="U3" t="n">
+        <v>-12.7625</v>
+      </c>
+      <c r="V3" t="n">
+        <v>-0.0017</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.0474</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.2053</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0766</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0707</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0863</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.0898</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.0524</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.1063</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0901</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0655</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.0892</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0211</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="R4" t="n">
+        <v>-0.0214</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.07729999999999999</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0747</v>
+      </c>
+      <c r="U4" t="n">
+        <v>-13.8705</v>
+      </c>
+      <c r="V4" t="n">
+        <v>-0.0017</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.0654</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.1793</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0464</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.1085</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.0207</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.1188</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.1091</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.1032</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.0596</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.0901</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.1085</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.0281</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.0213</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-0.0233</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.08409999999999999</v>
+      </c>
+      <c r="U5" t="n">
+        <v>-15.4195</v>
+      </c>
+      <c r="V5" t="n">
+        <v>-0.0017</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.0717</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.1375</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0446</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.0416</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0399</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.0377</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.0437</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.1269</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.1766</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.1221</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.0357</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.1161</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.1634</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.0186</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.0163</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.0109</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.0834</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-25.5255</v>
+      </c>
+      <c r="V6" t="n">
+        <v>-0.0017</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Overall = ROUND(intercept + sum(weight * rating) + DunkFlag weight * DunkFlag + height/weight terms), weights by Position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DunkFlag = 99 if Dunk &gt;= 75, 50 if Dunk &gt;= 60, else 0 (what build_roster writes to the record).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>The intercept already contains the neutral record bytes build_roster writes (B4F, B50, B55, ...).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Generated by scripts/overall_sheet.py from data/overall_model.json (LOO error 1.39, n=211). Edit the model via fit_overall.py, not here.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -16816,8 +18039,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF12"/>
+  <dimension ref="A1:AG12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -16980,6 +18206,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -17083,6 +18314,10 @@
       <c r="AF2" t="n">
         <v>2003185</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -17186,6 +18421,10 @@
       <c r="AF3" t="n">
         <v>2001580</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -17289,6 +18528,10 @@
       <c r="AF4" t="n">
         <v>56406</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -17392,6 +18635,10 @@
       <c r="AF5" t="n">
         <v>2003902</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -17495,6 +18742,10 @@
       <c r="AF6" t="n">
         <v>2001992</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -17598,6 +18849,10 @@
       <c r="AF7" t="n">
         <v>2003184</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17701,6 +18956,10 @@
       <c r="AF8" t="n">
         <v>2003183</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -17804,6 +19063,10 @@
       <c r="AF9" t="n">
         <v>2001541</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17907,6 +19170,10 @@
       <c r="AF10" t="n">
         <v>2001540</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -18010,6 +19277,10 @@
       <c r="AF11" t="n">
         <v>2000803</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -18112,6 +19383,10 @@
       </c>
       <c r="AF12" t="n">
         <v>2000797</v>
+      </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -18125,8 +19400,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF16"/>
+  <dimension ref="A1:AG16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -18289,6 +19567,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18392,6 +19675,10 @@
       <c r="AF2" t="n">
         <v>2004161</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18495,6 +19782,10 @@
       <c r="AF3" t="n">
         <v>2003164</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18598,6 +19889,10 @@
       <c r="AF4" t="n">
         <v>2004159</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18701,6 +19996,10 @@
       <c r="AF5" t="n">
         <v>2004160</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18804,6 +20103,10 @@
       <c r="AF6" t="n">
         <v>2004975</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18907,6 +20210,10 @@
       <c r="AF7" t="n">
         <v>2003165</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -19010,6 +20317,10 @@
       <c r="AF8" t="n">
         <v>2002073</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -19113,6 +20424,10 @@
       <c r="AF9" t="n">
         <v>2000514</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -19216,6 +20531,10 @@
       <c r="AF10" t="n">
         <v>2003110</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -19319,6 +20638,10 @@
       <c r="AF11" t="n">
         <v>2004162</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -19422,6 +20745,10 @@
       <c r="AF12" t="n">
         <v>2004971</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19525,6 +20852,10 @@
       <c r="AF13" t="n">
         <v>2004268</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19628,6 +20959,10 @@
       <c r="AF14" t="n">
         <v>2002027</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -19731,6 +21066,10 @@
       <c r="AF15" t="n">
         <v>2000305</v>
       </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -19833,6 +21172,10 @@
       </c>
       <c r="AF16" t="n">
         <v>2000309</v>
+      </c>
+      <c r="AG16">
+        <f>IF(ISNA(MATCH($C16,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L16:AD16,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*IF(Q16&gt;=75,99,IF(Q16&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*J16+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*K16,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -19846,8 +21189,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF15"/>
+  <dimension ref="A1:AG15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -20010,6 +21356,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -20113,6 +21464,10 @@
       <c r="AF2" t="n">
         <v>2001774</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -20216,6 +21571,10 @@
       <c r="AF3" t="n">
         <v>2003985</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -20319,6 +21678,10 @@
       <c r="AF4" t="n">
         <v>1400008</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -20422,6 +21785,10 @@
       <c r="AF5" t="n">
         <v>2003933</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -20525,6 +21892,10 @@
       <c r="AF6" t="n">
         <v>2001764</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -20628,6 +21999,10 @@
       <c r="AF7" t="n">
         <v>2003988</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -20731,6 +22106,10 @@
       <c r="AF8" t="n">
         <v>2001759</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -20834,6 +22213,10 @@
       <c r="AF9" t="n">
         <v>2003969</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -20937,6 +22320,10 @@
       <c r="AF10" t="n">
         <v>2003934</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -21040,6 +22427,10 @@
       <c r="AF11" t="n">
         <v>2001760</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -21143,6 +22534,10 @@
       <c r="AF12" t="n">
         <v>2003970</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -21246,6 +22641,10 @@
       <c r="AF13" t="n">
         <v>2001758</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -21349,6 +22748,10 @@
       <c r="AF14" t="n">
         <v>2001840</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -21451,6 +22854,10 @@
       </c>
       <c r="AF15" t="n">
         <v>2002957</v>
+      </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -21464,8 +22871,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF13"/>
+  <dimension ref="A1:AG13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -21628,6 +23038,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -21731,6 +23146,10 @@
       <c r="AF2" t="n">
         <v>2004673</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -21834,6 +23253,10 @@
       <c r="AF3" t="n">
         <v>2001905</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -21937,6 +23360,10 @@
       <c r="AF4" t="n">
         <v>2001908</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -22040,6 +23467,10 @@
       <c r="AF5" t="n">
         <v>2004677</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -22143,6 +23574,10 @@
       <c r="AF6" t="n">
         <v>2004675</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -22246,6 +23681,10 @@
       <c r="AF7" t="n">
         <v>2000441</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -22349,6 +23788,10 @@
       <c r="AF8" t="n">
         <v>2004987</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -22452,6 +23895,10 @@
       <c r="AF9" t="n">
         <v>2000439</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -22555,6 +24002,10 @@
       <c r="AF10" t="n">
         <v>2004674</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -22658,6 +24109,10 @@
       <c r="AF11" t="n">
         <v>2001911</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -22761,6 +24216,10 @@
       <c r="AF12" t="n">
         <v>2004682</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -22863,6 +24322,10 @@
       </c>
       <c r="AF13" t="n">
         <v>2004683</v>
+      </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -22876,8 +24339,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF13"/>
+  <dimension ref="A1:AG13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -23040,6 +24506,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -23143,6 +24614,10 @@
       <c r="AF2" t="n">
         <v>2003029</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -23246,6 +24721,10 @@
       <c r="AF3" t="n">
         <v>2004461</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -23349,6 +24828,10 @@
       <c r="AF4" t="n">
         <v>2004462</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -23452,6 +24935,10 @@
       <c r="AF5" t="n">
         <v>2004464</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -23555,6 +25042,10 @@
       <c r="AF6" t="n">
         <v>57676</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -23658,6 +25149,10 @@
       <c r="AF7" t="n">
         <v>2001575</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -23761,6 +25256,10 @@
       <c r="AF8" t="n">
         <v>2004463</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -23864,6 +25363,10 @@
       <c r="AF9" t="n">
         <v>6247</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -23967,6 +25470,10 @@
       <c r="AF10" t="n">
         <v>2001574</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -24070,6 +25577,10 @@
       <c r="AF11" t="n">
         <v>2000861</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -24173,6 +25684,10 @@
       <c r="AF12" t="n">
         <v>2004605</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -24275,6 +25790,10 @@
       </c>
       <c r="AF13" t="n">
         <v>2004603</v>
+      </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -24288,8 +25807,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF15"/>
+  <dimension ref="A1:AG15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -24452,6 +25974,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -24555,6 +26082,10 @@
       <c r="AF2" t="n">
         <v>2003864</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -24658,6 +26189,10 @@
       <c r="AF3" t="n">
         <v>2003168</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -24761,6 +26296,10 @@
       <c r="AF4" t="n">
         <v>2003170</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -24864,6 +26403,10 @@
       <c r="AF5" t="n">
         <v>2005235</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -24967,6 +26510,10 @@
       <c r="AF6" t="n">
         <v>2003178</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -25070,6 +26617,10 @@
       <c r="AF7" t="n">
         <v>2003169</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -25173,6 +26724,10 @@
       <c r="AF8" t="n">
         <v>2004273</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -25276,6 +26831,10 @@
       <c r="AF9" t="n">
         <v>2001472</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -25379,6 +26938,10 @@
       <c r="AF10" t="n">
         <v>2003862</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -25482,6 +27045,10 @@
       <c r="AF11" t="n">
         <v>2003107</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -25585,6 +27152,10 @@
       <c r="AF12" t="n">
         <v>2004275</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -25688,6 +27259,10 @@
       <c r="AF13" t="n">
         <v>2004274</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -25791,6 +27366,10 @@
       <c r="AF14" t="n">
         <v>2005213</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -25893,6 +27472,10 @@
       </c>
       <c r="AF15" t="n">
         <v>2004363</v>
+      </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -25906,8 +27489,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF15"/>
+  <dimension ref="A1:AG15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -26070,6 +27656,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -26173,6 +27764,10 @@
       <c r="AF2" t="n">
         <v>2001727</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -26276,6 +27871,10 @@
       <c r="AF3" t="n">
         <v>1400011</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -26379,6 +27978,10 @@
       <c r="AF4" t="n">
         <v>2004723</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -26482,6 +28085,10 @@
       <c r="AF5" t="n">
         <v>2004009</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -26585,6 +28192,10 @@
       <c r="AF6" t="n">
         <v>2004015</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -26688,6 +28299,10 @@
       <c r="AF7" t="n">
         <v>1400009</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -26791,6 +28406,10 @@
       <c r="AF8" t="n">
         <v>2004012</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -26894,6 +28513,10 @@
       <c r="AF9" t="n">
         <v>2004013</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -26997,6 +28620,10 @@
       <c r="AF10" t="n">
         <v>2005083</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -27100,6 +28727,10 @@
       <c r="AF11" t="n">
         <v>2002089</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -27203,6 +28834,10 @@
       <c r="AF12" t="n">
         <v>2004073</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -27306,6 +28941,10 @@
       <c r="AF13" t="n">
         <v>2004045</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -27409,6 +29048,10 @@
       <c r="AF14" t="n">
         <v>2004032</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -27511,6 +29154,10 @@
       </c>
       <c r="AF15" t="n">
         <v>2004011</v>
+      </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -27524,8 +29171,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF16"/>
+  <dimension ref="A1:AG16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="33" max="33"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -27688,6 +29338,11 @@
           <t>ProA ID</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -27791,6 +29446,10 @@
       <c r="AF2" t="n">
         <v>1400003</v>
       </c>
+      <c r="AG2">
+        <f>IF(ISNA(MATCH($C2,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L2:AD2,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*IF(Q2&gt;=75,99,IF(Q2&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*J2+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C2,'_Overall_Model'!$A$2:$A$6,0))*K2,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -27894,6 +29553,10 @@
       <c r="AF3" t="n">
         <v>1400007</v>
       </c>
+      <c r="AG3">
+        <f>IF(ISNA(MATCH($C3,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L3:AD3,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*IF(Q3&gt;=75,99,IF(Q3&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*J3+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C3,'_Overall_Model'!$A$2:$A$6,0))*K3,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -27997,6 +29660,10 @@
       <c r="AF4" t="n">
         <v>2004151</v>
       </c>
+      <c r="AG4">
+        <f>IF(ISNA(MATCH($C4,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L4:AD4,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*IF(Q4&gt;=75,99,IF(Q4&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*J4+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C4,'_Overall_Model'!$A$2:$A$6,0))*K4,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -28100,6 +29767,10 @@
       <c r="AF5" t="n">
         <v>2003855</v>
       </c>
+      <c r="AG5">
+        <f>IF(ISNA(MATCH($C5,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L5:AD5,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*IF(Q5&gt;=75,99,IF(Q5&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*J5+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C5,'_Overall_Model'!$A$2:$A$6,0))*K5,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -28203,6 +29874,10 @@
       <c r="AF6" t="n">
         <v>2003942</v>
       </c>
+      <c r="AG6">
+        <f>IF(ISNA(MATCH($C6,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L6:AD6,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*IF(Q6&gt;=75,99,IF(Q6&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*J6+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C6,'_Overall_Model'!$A$2:$A$6,0))*K6,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -28306,6 +29981,10 @@
       <c r="AF7" t="n">
         <v>2001623</v>
       </c>
+      <c r="AG7">
+        <f>IF(ISNA(MATCH($C7,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L7:AD7,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*IF(Q7&gt;=75,99,IF(Q7&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*J7+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C7,'_Overall_Model'!$A$2:$A$6,0))*K7,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -28409,6 +30088,10 @@
       <c r="AF8" t="n">
         <v>2003199</v>
       </c>
+      <c r="AG8">
+        <f>IF(ISNA(MATCH($C8,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L8:AD8,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*IF(Q8&gt;=75,99,IF(Q8&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*J8+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C8,'_Overall_Model'!$A$2:$A$6,0))*K8,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -28512,6 +30195,10 @@
       <c r="AF9" t="n">
         <v>1400028</v>
       </c>
+      <c r="AG9">
+        <f>IF(ISNA(MATCH($C9,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L9:AD9,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*IF(Q9&gt;=75,99,IF(Q9&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*J9+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C9,'_Overall_Model'!$A$2:$A$6,0))*K9,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -28615,6 +30302,10 @@
       <c r="AF10" t="n">
         <v>2003858</v>
       </c>
+      <c r="AG10">
+        <f>IF(ISNA(MATCH($C10,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L10:AD10,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*IF(Q10&gt;=75,99,IF(Q10&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*J10+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C10,'_Overall_Model'!$A$2:$A$6,0))*K10,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -28718,6 +30409,10 @@
       <c r="AF11" t="n">
         <v>2001288</v>
       </c>
+      <c r="AG11">
+        <f>IF(ISNA(MATCH($C11,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L11:AD11,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*IF(Q11&gt;=75,99,IF(Q11&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*J11+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C11,'_Overall_Model'!$A$2:$A$6,0))*K11,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -28821,6 +30516,10 @@
       <c r="AF12" t="n">
         <v>2001627</v>
       </c>
+      <c r="AG12">
+        <f>IF(ISNA(MATCH($C12,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L12:AD12,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*IF(Q12&gt;=75,99,IF(Q12&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*J12+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C12,'_Overall_Model'!$A$2:$A$6,0))*K12,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -28924,6 +30623,10 @@
       <c r="AF13" t="n">
         <v>1400014</v>
       </c>
+      <c r="AG13">
+        <f>IF(ISNA(MATCH($C13,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L13:AD13,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*IF(Q13&gt;=75,99,IF(Q13&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*J13+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C13,'_Overall_Model'!$A$2:$A$6,0))*K13,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -29027,6 +30730,10 @@
       <c r="AF14" t="n">
         <v>2001622</v>
       </c>
+      <c r="AG14">
+        <f>IF(ISNA(MATCH($C14,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L14:AD14,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*IF(Q14&gt;=75,99,IF(Q14&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*J14+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C14,'_Overall_Model'!$A$2:$A$6,0))*K14,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -29130,6 +30837,10 @@
       <c r="AF15" t="n">
         <v>2001626</v>
       </c>
+      <c r="AG15">
+        <f>IF(ISNA(MATCH($C15,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L15:AD15,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*IF(Q15&gt;=75,99,IF(Q15&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*J15+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C15,'_Overall_Model'!$A$2:$A$6,0))*K15,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -29232,6 +30943,10 @@
       </c>
       <c r="AF16" t="n">
         <v>6604</v>
+      </c>
+      <c r="AG16">
+        <f>IF(ISNA(MATCH($C16,'_Overall_Model'!$A$2:$A$6,0)),"",ROUND(SUMPRODUCT(L16:AD16,INDEX('_Overall_Model'!$B$2:$T$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0),0))+INDEX('_Overall_Model'!$U$2:$U$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))+INDEX('_Overall_Model'!$V$2:$V$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*IF(Q16&gt;=75,99,IF(Q16&gt;=60,50,0))+INDEX('_Overall_Model'!$W$2:$W$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*J16+INDEX('_Overall_Model'!$X$2:$X$6,MATCH($C16,'_Overall_Model'!$A$2:$A$6,0))*K16,0))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>